<commit_message>
changed and worked on the finaloutput
</commit_message>
<xml_diff>
--- a/script2/finaloutput.xlsx
+++ b/script2/finaloutput.xlsx
@@ -22576,7 +22576,7 @@
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>Xiaomi Xiaomi Vacuum Cleaner Mi Robot G30 Max Filter Kit EU BHR08C4GL</t>
         </is>
       </c>
       <c r="E715" t="n">
@@ -26329,7 +26329,7 @@
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>Kitchenaid</t>
+          <t>Kitchenaid 5KEK1701EPL Electric Kettle</t>
         </is>
       </c>
       <c r="E836" t="n">
@@ -26856,7 +26856,7 @@
       </c>
       <c r="D853" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens VZ41AFP Staubsaugerbeutel</t>
         </is>
       </c>
       <c r="E853" t="n">
@@ -26949,7 +26949,7 @@
       </c>
       <c r="D856" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HEZ431002 Backblech</t>
         </is>
       </c>
       <c r="E856" t="n">
@@ -26980,7 +26980,7 @@
       </c>
       <c r="D857" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HEZ634000</t>
         </is>
       </c>
       <c r="E857" t="n">
@@ -27011,7 +27011,7 @@
       </c>
       <c r="D858" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WMZ2381 Verlängerung Wasserzulaufschlauch</t>
         </is>
       </c>
       <c r="E858" t="n">
@@ -27197,7 +27197,7 @@
       </c>
       <c r="D864" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch TWK4P440 DesignLine</t>
         </is>
       </c>
       <c r="E864" t="n">
@@ -27321,7 +27321,7 @@
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje BM201SG3BG  Mikrowelle mit Grill Schwarz</t>
         </is>
       </c>
       <c r="E868" t="n">
@@ -27352,7 +27352,7 @@
       </c>
       <c r="D869" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI6401BX Kochfeld Induktion 60 cm autark</t>
         </is>
       </c>
       <c r="E869" t="n">
@@ -27445,7 +27445,7 @@
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RB49CPW</t>
         </is>
       </c>
       <c r="E872" t="n">
@@ -27476,7 +27476,7 @@
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RB49CPW Kühlschrank mit Gefrierfach Stand</t>
         </is>
       </c>
       <c r="E873" t="n">
@@ -27569,7 +27569,7 @@
       </c>
       <c r="D876" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens LB55565 Lüfterbaustein Silbermetallic</t>
         </is>
       </c>
       <c r="E876" t="n">
@@ -27662,7 +27662,7 @@
       </c>
       <c r="D879" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WPNF5A84A2TS/AT Waschmaschine Stand 60 cm 8 kg</t>
         </is>
       </c>
       <c r="E879" t="n">
@@ -27693,7 +27693,7 @@
       </c>
       <c r="D880" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI642E90X Geschirrspüler einbau 60cm teilintegriert</t>
         </is>
       </c>
       <c r="E880" t="n">
@@ -27724,7 +27724,7 @@
       </c>
       <c r="D881" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW80FG3M05AWEG Waschmaschine 8kg 1400 U/min</t>
         </is>
       </c>
       <c r="E881" t="n">
@@ -27786,7 +27786,7 @@
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens LC67BIP50 Wand-Esse Edelstahl 60 cm</t>
         </is>
       </c>
       <c r="E883" t="n">
@@ -27817,7 +27817,7 @@
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RL481N4BIE Kühlschrank Stand Inox-Look</t>
         </is>
       </c>
       <c r="E884" t="n">
@@ -27910,7 +27910,7 @@
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje JUMP SET AQUA/C  BackofenSet Einbau 60 cm schwarz</t>
         </is>
       </c>
       <c r="E887" t="n">
@@ -27941,7 +27941,7 @@
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje NRB620C61X4WFE Kühl-Gefrierkombination Stand</t>
         </is>
       </c>
       <c r="E888" t="n">
@@ -28034,7 +28034,7 @@
       </c>
       <c r="D891" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WD2PA964ADW/AT Waschtrockner 9 kg Waschen 6 kg Trocknen</t>
         </is>
       </c>
       <c r="E891" t="n">
@@ -28065,7 +28065,7 @@
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens EI645CFB6E  Induktions-Kochfeld, 60 cm herdgebunden</t>
         </is>
       </c>
       <c r="E892" t="n">
@@ -28127,7 +28127,7 @@
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko HSM46740 Gefriertruhe  451 l</t>
         </is>
       </c>
       <c r="E894" t="n">
@@ -28158,7 +28158,7 @@
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch KÜHLSCHRANK INTEG.**** 88X56CM</t>
         </is>
       </c>
       <c r="E895" t="n">
@@ -28189,7 +28189,7 @@
       </c>
       <c r="D896" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG LAVAMAT L6FBA50490 Waschmaschine Frontlader 9kg</t>
         </is>
       </c>
       <c r="E896" t="n">
@@ -28220,7 +28220,7 @@
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FAVORIT FSE73427P</t>
         </is>
       </c>
       <c r="E897" t="n">
@@ -28251,7 +28251,7 @@
       </c>
       <c r="D898" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SBI4ECS28E Geschirrspüler Einbau teilintegriert 60 cm XXL</t>
         </is>
       </c>
       <c r="E898" t="n">
@@ -28375,7 +28375,7 @@
       </c>
       <c r="D902" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FSK74747P</t>
         </is>
       </c>
       <c r="E902" t="n">
@@ -28406,7 +28406,7 @@
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WASCHVOLLAUTOMAT 9KG 1400UMIN</t>
         </is>
       </c>
       <c r="E903" t="n">
@@ -28437,7 +28437,7 @@
       </c>
       <c r="D904" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW11DB7B94GEU3 Waschmaschine 11 kg 1400U/Min A-20%</t>
         </is>
       </c>
       <c r="E904" t="n">
@@ -28468,7 +28468,7 @@
       </c>
       <c r="D905" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WGB244071 Waschmaschine Weiß 9 kg 1400 U/min</t>
         </is>
       </c>
       <c r="E905" t="n">
@@ -28499,7 +28499,7 @@
       </c>
       <c r="D906" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens HE578BBS3 iQ500, Einbau-Herd, 60 x 60 cm,</t>
         </is>
       </c>
       <c r="E906" t="n">
@@ -28654,7 +28654,7 @@
       </c>
       <c r="D911" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RQ760N4SASE Side by Side mit Wassertank</t>
         </is>
       </c>
       <c r="E911" t="n">
@@ -28778,7 +28778,7 @@
       </c>
       <c r="D915" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS68CG852DS9EF Side by Side mit Wassertank NoFrost</t>
         </is>
       </c>
       <c r="E915" t="n">
@@ -28809,7 +28809,7 @@
       </c>
       <c r="D916" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS80F65KDFEF Side-by-Side  NoFrost 640 Liter</t>
         </is>
       </c>
       <c r="E916" t="n">
@@ -28871,7 +28871,7 @@
       </c>
       <c r="D918" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung SSD 9100 PRO NVMe 8TB Heatsink</t>
         </is>
       </c>
       <c r="E918" t="n">
@@ -29057,7 +29057,7 @@
       </c>
       <c r="D924" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG DPGR-AP1 Brat- und Fettpfanne</t>
         </is>
       </c>
       <c r="E924" t="n">
@@ -29243,7 +29243,7 @@
       </c>
       <c r="D930" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung NK24N1331IS Dunstabzugshaube 60cm Edelstahl</t>
         </is>
       </c>
       <c r="E930" t="n">
@@ -29305,7 +29305,7 @@
       </c>
       <c r="D932" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WHT6SYB Dekorativ Dunstabzug Kamin 60cm Schwarz</t>
         </is>
       </c>
       <c r="E932" t="n">
@@ -29491,7 +29491,7 @@
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens ET601FNP1E Einbau Flächenbündiges Design</t>
         </is>
       </c>
       <c r="E938" t="n">
@@ -29522,7 +29522,7 @@
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDIN36432 Geschirrspüler Einbau 60 cm vollintegriert</t>
         </is>
       </c>
       <c r="E939" t="n">
@@ -29553,7 +29553,7 @@
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje F49CPW</t>
         </is>
       </c>
       <c r="E940" t="n">
@@ -29584,7 +29584,7 @@
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BM3WFT38413W Waschmaschine 1400 U/min 8 kg</t>
         </is>
       </c>
       <c r="E941" t="n">
@@ -29646,7 +29646,7 @@
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko B5WFU58416W</t>
         </is>
       </c>
       <c r="E943" t="n">
@@ -29677,7 +29677,7 @@
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG L6FBC41480  LAVAMAT Waschmaschinen Frontlader Weiss</t>
         </is>
       </c>
       <c r="E944" t="n">
@@ -29708,7 +29708,7 @@
       </c>
       <c r="D945" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPV2HKX42E Geschirrspüler Einbau 45 cm vollintegriert</t>
         </is>
       </c>
       <c r="E945" t="n">
@@ -29770,7 +29770,7 @@
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HBG578BS3 Backofen Edelstahl Schwarz</t>
         </is>
       </c>
       <c r="E947" t="n">
@@ -29801,7 +29801,7 @@
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FSE73407P</t>
         </is>
       </c>
       <c r="E948" t="n">
@@ -29832,7 +29832,7 @@
       </c>
       <c r="D949" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FEE7341AZM</t>
         </is>
       </c>
       <c r="E949" t="n">
@@ -29863,7 +29863,7 @@
       </c>
       <c r="D950" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch KIV86NSE0 Kühl-/Gefrierkombinationen Einbau Weiss</t>
         </is>
       </c>
       <c r="E950" t="n">
@@ -29894,7 +29894,7 @@
       </c>
       <c r="D951" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMI6ECS12E Teilintegrierter Geschirrspüler, 60 cm, Edelstahl</t>
         </is>
       </c>
       <c r="E951" t="n">
@@ -29925,7 +29925,7 @@
       </c>
       <c r="D952" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch CBG7341B1 Kompaktbackofen 60x45 EEK: A+</t>
         </is>
       </c>
       <c r="E952" t="n">
@@ -29987,7 +29987,7 @@
       </c>
       <c r="D954" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch ATMKHERD2 (HEA2130B3 + NKN64RGA2E) Herdset Einbau</t>
         </is>
       </c>
       <c r="E954" t="n">
@@ -30142,7 +30142,7 @@
       </c>
       <c r="D959" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung QE65S85F 65 Zoll 4K Vision AI TV; OLED TV Schwarz Fernseher</t>
         </is>
       </c>
       <c r="E959" t="n">
@@ -30204,7 +30204,7 @@
       </c>
       <c r="D961" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS90F64EDFEF Side-by-Side  Premium Black Steel</t>
         </is>
       </c>
       <c r="E961" t="n">
@@ -30545,7 +30545,7 @@
       </c>
       <c r="D972" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung Sonic the Hedgehog microSDXC 512GB</t>
         </is>
       </c>
       <c r="E972" t="n">
@@ -30700,7 +30700,7 @@
       </c>
       <c r="D977" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens FF023LMB2 iQ300 Mikrowelle</t>
         </is>
       </c>
       <c r="E977" t="n">
@@ -30762,7 +30762,7 @@
       </c>
       <c r="D979" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BBIMA13300XS Backofen AirFry 60 cm Schwarz</t>
         </is>
       </c>
       <c r="E979" t="n">
@@ -30855,7 +30855,7 @@
       </c>
       <c r="D982" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BSA65334ABDG Einbaubackofen schwarz 77 Liter</t>
         </is>
       </c>
       <c r="E982" t="n">
@@ -30886,7 +30886,7 @@
       </c>
       <c r="D983" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GV663A66  Einbau Geschirrspüler 60cm vollintegriert</t>
         </is>
       </c>
       <c r="E983" t="n">
@@ -30948,7 +30948,7 @@
       </c>
       <c r="D985" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMS2ITW33E Serie 2 Freistehender Geschirrspüler 60 cm</t>
         </is>
       </c>
       <c r="E985" t="n">
@@ -30979,7 +30979,7 @@
       </c>
       <c r="D986" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI673B90X Geschirrspüler Einbau 60cm teilintegriert</t>
         </is>
       </c>
       <c r="E986" t="n">
@@ -31041,7 +31041,7 @@
       </c>
       <c r="D988" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDDN38440XD</t>
         </is>
       </c>
       <c r="E988" t="n">
@@ -31103,7 +31103,7 @@
       </c>
       <c r="D990" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch GESCHIRRSPÜLER VOLLI.     60CM</t>
         </is>
       </c>
       <c r="E990" t="n">
@@ -31134,7 +31134,7 @@
       </c>
       <c r="D991" t="inlineStr">
         <is>
-          <t>Electrolux</t>
+          <t>Electrolux LXB3AE82R</t>
         </is>
       </c>
       <c r="E991" t="n">
@@ -31165,7 +31165,7 @@
       </c>
       <c r="D992" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch KIR21ADD1 Serie 6 Einbau-Kühlschrank ohne Gefrierfach, 88cm</t>
         </is>
       </c>
       <c r="E992" t="n">
@@ -31196,7 +31196,7 @@
       </c>
       <c r="D993" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje Steel Set 4  BCS6737E06X +  ECD634BCSC</t>
         </is>
       </c>
       <c r="E993" t="n">
@@ -31227,7 +31227,7 @@
       </c>
       <c r="D994" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens GESCHIRRSPÜLER INTEG.     60CM</t>
         </is>
       </c>
       <c r="E994" t="n">
@@ -31258,7 +31258,7 @@
       </c>
       <c r="D995" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG LAVAMAT L6FBA51680 Waschmaschine 8 kg 1600 U/min</t>
         </is>
       </c>
       <c r="E995" t="n">
@@ -31289,7 +31289,7 @@
       </c>
       <c r="D996" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPÜLER TEILINTEGRIERT 60CM</t>
         </is>
       </c>
       <c r="E996" t="n">
@@ -31320,7 +31320,7 @@
       </c>
       <c r="D997" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SR53HS74KE Geschirrspüler Einbau 45cm teilintegriert</t>
         </is>
       </c>
       <c r="E997" t="n">
@@ -31475,7 +31475,7 @@
       </c>
       <c r="D1002" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WF90F09C4SU3 AI Waschmaschine 9kg 1400 U/min</t>
         </is>
       </c>
       <c r="E1002" t="n">
@@ -31537,7 +31537,7 @@
       </c>
       <c r="D1004" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KG39N2XAG Küh-Gefrierkombination  BlackSteel NoFrost</t>
         </is>
       </c>
       <c r="E1004" t="n">
@@ -31568,7 +31568,7 @@
       </c>
       <c r="D1005" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KI77SXFE0 iQ500, Einbau-Kühl-Gefrier-Kombination</t>
         </is>
       </c>
       <c r="E1005" t="n">
@@ -31599,7 +31599,7 @@
       </c>
       <c r="D1006" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RQ5P605NSVE Multi Door Side-By-Side (4Tür) 591Liter</t>
         </is>
       </c>
       <c r="E1006" t="n">
@@ -31661,7 +31661,7 @@
       </c>
       <c r="D1008" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch Bosch Siemens Neff ORIGINAL Lampe  Blau</t>
         </is>
       </c>
       <c r="E1008" t="n">
@@ -31847,7 +31847,7 @@
       </c>
       <c r="D1014" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG DUB1611M</t>
         </is>
       </c>
       <c r="E1014" t="n">
@@ -31878,7 +31878,7 @@
       </c>
       <c r="D1015" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko CTB 9250 XH Flachschirmhaube Einbau Edelstahl</t>
         </is>
       </c>
       <c r="E1015" t="n">
@@ -32035,7 +32035,7 @@
       </c>
       <c r="D1020" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDFN26441W Geschirspüler Stand 6 Programme</t>
         </is>
       </c>
       <c r="E1020" t="n">
@@ -32159,7 +32159,7 @@
       </c>
       <c r="D1024" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 55A6Q</t>
         </is>
       </c>
       <c r="E1024" t="n">
@@ -32190,7 +32190,7 @@
       </c>
       <c r="D1025" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje NFB612CSXL4  Kühl-Gefrierkombination Stand Nofrost</t>
         </is>
       </c>
       <c r="E1025" t="n">
@@ -32283,7 +32283,7 @@
       </c>
       <c r="D1028" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje Jump Induction Set 2 Backofen Set</t>
         </is>
       </c>
       <c r="E1028" t="n">
@@ -32314,7 +32314,7 @@
       </c>
       <c r="D1029" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HBA3140B3 Backofen Schwarz 3D Heißluft</t>
         </is>
       </c>
       <c r="E1029" t="n">
@@ -32345,7 +32345,7 @@
       </c>
       <c r="D1030" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense WF5i1245BWR Waschmaschine 12 kg 1400 U/Min.</t>
         </is>
       </c>
       <c r="E1030" t="n">
@@ -32376,7 +32376,7 @@
       </c>
       <c r="D1031" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SR43ES25ME Unterbau-Einbau Geschirrspüler 45 cm</t>
         </is>
       </c>
       <c r="E1031" t="n">
@@ -32407,7 +32407,7 @@
       </c>
       <c r="D1032" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WAN2820EP Waschmaschine Stand 60 cm weiß</t>
         </is>
       </c>
       <c r="E1032" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="D1033" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG TO64RAF7XB</t>
         </is>
       </c>
       <c r="E1033" t="n">
@@ -32531,7 +32531,7 @@
       </c>
       <c r="D1036" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WUU28T48  8kg Frontlader Waschmaschine unterbaufähig</t>
         </is>
       </c>
       <c r="E1036" t="n">
@@ -32562,7 +32562,7 @@
       </c>
       <c r="D1037" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko B7T692A3WW  Wärmepumpentrockner 9kg</t>
         </is>
       </c>
       <c r="E1037" t="n">
@@ -32593,7 +32593,7 @@
       </c>
       <c r="D1038" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RL5K370GSFC Kühlschrank Stand 372l, Schwarz</t>
         </is>
       </c>
       <c r="E1038" t="n">
@@ -32624,7 +32624,7 @@
       </c>
       <c r="D1039" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SN53ES22AE Geschirrspüler Einbau teilintegriert 60 cm</t>
         </is>
       </c>
       <c r="E1039" t="n">
@@ -32655,7 +32655,7 @@
       </c>
       <c r="D1040" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens BE732R1B1  iQ700 Einbau-Mikrowelle Schwarz Edelstahl</t>
         </is>
       </c>
       <c r="E1040" t="n">
@@ -32686,7 +32686,7 @@
       </c>
       <c r="D1041" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KI42LVFE0 Kühlschrank Einbau 122cm Nische Weiß</t>
         </is>
       </c>
       <c r="E1041" t="n">
@@ -32779,7 +32779,7 @@
       </c>
       <c r="D1044" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S27FG810SU - G81SF Series - OLED-Monitor - Gaming - 68.6 cm</t>
         </is>
       </c>
       <c r="E1044" t="n">
@@ -32872,7 +32872,7 @@
       </c>
       <c r="D1047" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMI4ECS28E Geschirrspüler Einbau teilintegriert 60 cm</t>
         </is>
       </c>
       <c r="E1047" t="n">
@@ -33244,7 +33244,7 @@
       </c>
       <c r="D1059" t="inlineStr">
         <is>
-          <t>Electrolux</t>
+          <t>Electrolux KRB2AE88S</t>
         </is>
       </c>
       <c r="E1059" t="n">
@@ -33275,7 +33275,7 @@
       </c>
       <c r="D1060" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDSA250K4SN Einbau Kühl-Gefrierkombination 220 Liter</t>
         </is>
       </c>
       <c r="E1060" t="n">
@@ -33337,7 +33337,7 @@
       </c>
       <c r="D1062" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPV2HMX42E Geschirrspüler Einbau vollintegriert 45 cm</t>
         </is>
       </c>
       <c r="E1062" t="n">
@@ -33399,7 +33399,7 @@
       </c>
       <c r="D1064" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW90DG5G34AEEG Waschmaschine Slim 9kg ,1400 U/min, 48cm Tief</t>
         </is>
       </c>
       <c r="E1064" t="n">
@@ -33430,7 +33430,7 @@
       </c>
       <c r="D1065" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW1EDG5B25AEEG  Waschmaschine 11 kg 1400 U/min</t>
         </is>
       </c>
       <c r="E1065" t="n">
@@ -33492,7 +33492,7 @@
       </c>
       <c r="D1067" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 75E7NQ PRO  75 '' E7N PRO | QLED Smart TV 4K 144 Hz</t>
         </is>
       </c>
       <c r="E1067" t="n">
@@ -33554,7 +33554,7 @@
       </c>
       <c r="D1069" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG WASCHMASCHINE TOPL. 6KG  1300U</t>
         </is>
       </c>
       <c r="E1069" t="n">
@@ -33585,7 +33585,7 @@
       </c>
       <c r="D1070" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SR65ZX22ME Geschirrspüler Einbau vollintegriert 45cm</t>
         </is>
       </c>
       <c r="E1070" t="n">
@@ -33616,7 +33616,7 @@
       </c>
       <c r="D1071" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens EX801KYW1E Einbau Induktion 80cm Edelstahl</t>
         </is>
       </c>
       <c r="E1071" t="n">
@@ -33678,7 +33678,7 @@
       </c>
       <c r="D1073" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F64KETEF Side by Side Nofrost  640Liter</t>
         </is>
       </c>
       <c r="E1073" t="n">
@@ -33709,7 +33709,7 @@
       </c>
       <c r="D1074" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung COLOR E-PAPER DISPLAY 32ZOLL</t>
         </is>
       </c>
       <c r="E1074" t="n">
@@ -33771,7 +33771,7 @@
       </c>
       <c r="D1076" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>LG OLED83C54LA  4K OLED evo Smart TV Fernseher</t>
         </is>
       </c>
       <c r="E1076" t="n">
@@ -33802,7 +33802,7 @@
       </c>
       <c r="D1077" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG STAUBBEUTEL F. VAMPYR 5000+</t>
         </is>
       </c>
       <c r="E1077" t="n">
@@ -33833,7 +33833,7 @@
       </c>
       <c r="D1078" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje M882528 Filter für WHU</t>
         </is>
       </c>
       <c r="E1078" t="n">
@@ -33864,7 +33864,7 @@
       </c>
       <c r="D1079" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje T850DPB Toaster</t>
         </is>
       </c>
       <c r="E1079" t="n">
@@ -34050,7 +34050,7 @@
       </c>
       <c r="D1085" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje BHI611ES Lüfterbaustein Montage in Oberschrank</t>
         </is>
       </c>
       <c r="E1085" t="n">
@@ -34081,7 +34081,7 @@
       </c>
       <c r="D1086" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje ECT322BCSC/BCSP  Kochfeld 30cm Autark</t>
         </is>
       </c>
       <c r="E1086" t="n">
@@ -34112,7 +34112,7 @@
       </c>
       <c r="D1087" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens LU62LFA21 60 cm Weiß   Unterbauhaube</t>
         </is>
       </c>
       <c r="E1087" t="n">
@@ -34143,7 +34143,7 @@
       </c>
       <c r="D1088" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI601FMC Induktionskochfeld 60cm autark</t>
         </is>
       </c>
       <c r="E1088" t="n">
@@ -34267,7 +34267,7 @@
       </c>
       <c r="D1092" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GE5A23WH Stand Herd  50cm</t>
         </is>
       </c>
       <c r="E1092" t="n">
@@ -34391,7 +34391,7 @@
       </c>
       <c r="D1096" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch BSS825ALL Unlimited Gen2 Akku-Staubsauger Weiß</t>
         </is>
       </c>
       <c r="E1096" t="n">
@@ -34484,7 +34484,7 @@
       </c>
       <c r="D1099" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch PKM675DP1D Kochstelle Glaskeramik 60 cm</t>
         </is>
       </c>
       <c r="E1099" t="n">
@@ -34515,7 +34515,7 @@
       </c>
       <c r="D1100" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch MIKROWELLE EINBAU 800W 39X50CM</t>
         </is>
       </c>
       <c r="E1100" t="n">
@@ -34577,7 +34577,7 @@
       </c>
       <c r="D1102" t="inlineStr">
         <is>
-          <t>Electrolux</t>
+          <t>Electrolux LUB3AE88S</t>
         </is>
       </c>
       <c r="E1102" t="n">
@@ -34608,7 +34608,7 @@
       </c>
       <c r="D1103" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG TSK5O88WDF  Kühlschrank Einbau</t>
         </is>
       </c>
       <c r="E1103" t="n">
@@ -34670,7 +34670,7 @@
       </c>
       <c r="D1105" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG TSF5O88WDF</t>
         </is>
       </c>
       <c r="E1105" t="n">
@@ -34701,7 +34701,7 @@
       </c>
       <c r="D1106" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens WQ45B2B40  iQ700, Wärmepumpen-Trockner, 9 kg</t>
         </is>
       </c>
       <c r="E1106" t="n">
@@ -34732,7 +34732,7 @@
       </c>
       <c r="D1107" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung LS49CG950EUXEN Odyssey Gaming Monitor G95C (49'')</t>
         </is>
       </c>
       <c r="E1107" t="n">
@@ -34763,7 +34763,7 @@
       </c>
       <c r="D1108" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung DV90DB7845GEU3  Wärmepumpentrockner 9 kg</t>
         </is>
       </c>
       <c r="E1108" t="n">
@@ -34825,7 +34825,7 @@
       </c>
       <c r="D1110" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RF50C530EB1 French Door mit AI NoFrost</t>
         </is>
       </c>
       <c r="E1110" t="n">
@@ -34856,7 +34856,7 @@
       </c>
       <c r="D1111" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WRB247C40 Wärmepumpentrockner 9kg</t>
         </is>
       </c>
       <c r="E1111" t="n">
@@ -34887,7 +34887,7 @@
       </c>
       <c r="D1112" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F64KDTEF Side by Side NoFrost 640 Liter</t>
         </is>
       </c>
       <c r="E1112" t="n">
@@ -34918,7 +34918,7 @@
       </c>
       <c r="D1113" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F64KDFEF Side by Side NoFrost 640 Liter</t>
         </is>
       </c>
       <c r="E1113" t="n">
@@ -35042,7 +35042,7 @@
       </c>
       <c r="D1117" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje H23MOBSD1HG Mikrowelle mit Grill,23Liter Schwarz</t>
         </is>
       </c>
       <c r="E1117" t="n">
@@ -35104,7 +35104,7 @@
       </c>
       <c r="D1119" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje EC321BCSC Elektrokochfeld 30cm domino</t>
         </is>
       </c>
       <c r="E1119" t="n">
@@ -35197,7 +35197,7 @@
       </c>
       <c r="D1122" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDSN26440X Geschirrspüler EInbau teilintegriert 60 cm</t>
         </is>
       </c>
       <c r="E1122" t="n">
@@ -35228,7 +35228,7 @@
       </c>
       <c r="D1123" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RK418DPS4WD Kühl-/Gefrierkombination Stand</t>
         </is>
       </c>
       <c r="E1123" t="n">
@@ -35259,7 +35259,7 @@
       </c>
       <c r="D1124" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens HB517GBS3 iQ500, Einbau-Backofen, 60 x 60 cm</t>
         </is>
       </c>
       <c r="E1124" t="n">
@@ -35352,7 +35352,7 @@
       </c>
       <c r="D1127" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens HE578GBS3 iQ500, Einbau-Herd, 60 x 60 cm,</t>
         </is>
       </c>
       <c r="E1127" t="n">
@@ -35414,7 +35414,7 @@
       </c>
       <c r="D1129" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S49DG934SU - G93SD Series - OLED-Monitor - Gaming - gebog</t>
         </is>
       </c>
       <c r="E1129" t="n">
@@ -35569,7 +35569,7 @@
       </c>
       <c r="D1134" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG NRN64A06XB</t>
         </is>
       </c>
       <c r="E1134" t="n">
@@ -35631,7 +35631,7 @@
       </c>
       <c r="D1136" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HS673A90W Geschirrspüler Stand 60 cm Weiss</t>
         </is>
       </c>
       <c r="E1136" t="n">
@@ -35662,7 +35662,7 @@
       </c>
       <c r="D1137" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BSA66334PBDG Einbaubackofen 60cm</t>
         </is>
       </c>
       <c r="E1137" t="n">
@@ -35755,7 +35755,7 @@
       </c>
       <c r="D1140" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BI614P8B Einbaubackofen 60cm</t>
         </is>
       </c>
       <c r="E1140" t="n">
@@ -35910,7 +35910,7 @@
       </c>
       <c r="D1145" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KU21RVFE0 Kühlschrank Einbau-Unterbau 82 x 59.8 cm</t>
         </is>
       </c>
       <c r="E1145" t="n">
@@ -35972,7 +35972,7 @@
       </c>
       <c r="D1147" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WGG256F7AT Serie 6 Waschmaschine 10 kg, 1600 U/min</t>
         </is>
       </c>
       <c r="E1147" t="n">
@@ -36096,7 +36096,7 @@
       </c>
       <c r="D1151" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate microSDXC 256GB</t>
         </is>
       </c>
       <c r="E1151" t="n">
@@ -36127,7 +36127,7 @@
       </c>
       <c r="D1152" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje W3NGPI72SBS/AT</t>
         </is>
       </c>
       <c r="E1152" t="n">
@@ -36189,7 +36189,7 @@
       </c>
       <c r="D1154" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RI517E41WF Kühlschrank Einbau 178cm Weiss</t>
         </is>
       </c>
       <c r="E1154" t="n">
@@ -36220,7 +36220,7 @@
       </c>
       <c r="D1155" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung BRD27713EWW Kühlschrank mit Gefrierfach Festtür 178cm Nische</t>
         </is>
       </c>
       <c r="E1155" t="n">
@@ -36251,7 +36251,7 @@
       </c>
       <c r="D1156" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RBI418EE0 Kühlschrank Einbau mit Gefrierfach  178cm Nische</t>
         </is>
       </c>
       <c r="E1156" t="n">
@@ -36623,7 +36623,7 @@
       </c>
       <c r="D1168" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje R49CPW Kühlschrank Stand 56cm breit</t>
         </is>
       </c>
       <c r="E1168" t="n">
@@ -36654,7 +36654,7 @@
       </c>
       <c r="D1169" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDSS25N20X Geschirrspüler Einbau 45 cm edeltstahl</t>
         </is>
       </c>
       <c r="E1169" t="n">
@@ -36716,7 +36716,7 @@
       </c>
       <c r="D1171" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPÜLER TEILINTEGRIERT     60CM</t>
         </is>
       </c>
       <c r="E1171" t="n">
@@ -36747,7 +36747,7 @@
       </c>
       <c r="D1172" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BFS615S8B  Dampfbackofen Einbau</t>
         </is>
       </c>
       <c r="E1172" t="n">
@@ -36840,7 +36840,7 @@
       </c>
       <c r="D1175" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG M3OCD301 Entkalker für Dampfbacköfen 250ml</t>
         </is>
       </c>
       <c r="E1175" t="n">
@@ -36964,7 +36964,7 @@
       </c>
       <c r="D1179" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RBIU609DA1 Unterbau-Einbau Kühlschrank mit Gefrierfach</t>
         </is>
       </c>
       <c r="E1179" t="n">
@@ -36995,7 +36995,7 @@
       </c>
       <c r="D1180" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WPNEI84A1DTS Waschmaschine 8kg 1400 U/min</t>
         </is>
       </c>
       <c r="E1180" t="n">
@@ -37119,7 +37119,7 @@
       </c>
       <c r="D1184" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BAS614P8B Einbau Backofen mit Dampffunktion</t>
         </is>
       </c>
       <c r="E1184" t="n">
@@ -37150,7 +37150,7 @@
       </c>
       <c r="D1185" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WASCHMASCHINE 1400UPM 7KG 60CM</t>
         </is>
       </c>
       <c r="E1185" t="n">
@@ -37336,7 +37336,7 @@
       </c>
       <c r="D1191" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S27D800EAU - S80D Series - LED-Monitor - 68 cm (27")</t>
         </is>
       </c>
       <c r="E1191" t="n">
@@ -37398,7 +37398,7 @@
       </c>
       <c r="D1193" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HV693A65UVAD  Geschirrspüler vollintegriert 60 cm</t>
         </is>
       </c>
       <c r="E1193" t="n">
@@ -37460,7 +37460,7 @@
       </c>
       <c r="D1195" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WD81TA049BE/EG Waschtrockner 8 kg Waschen 5 kg Trocknen</t>
         </is>
       </c>
       <c r="E1195" t="n">
@@ -37522,7 +37522,7 @@
       </c>
       <c r="D1197" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WAN28094 Waschmaschine 8kg 1400 U/min Weiss</t>
         </is>
       </c>
       <c r="E1197" t="n">
@@ -37553,7 +37553,7 @@
       </c>
       <c r="D1198" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch PXX675DC1E Induktionskochfeld Autark 60 cm</t>
         </is>
       </c>
       <c r="E1198" t="n">
@@ -37646,7 +37646,7 @@
       </c>
       <c r="D1201" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung DV90F09F4SU3  AI Wärmepumpentrockner 9 kg</t>
         </is>
       </c>
       <c r="E1201" t="n">
@@ -37708,7 +37708,7 @@
       </c>
       <c r="D1203" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje B6128B</t>
         </is>
       </c>
       <c r="E1203" t="n">
@@ -37770,7 +37770,7 @@
       </c>
       <c r="D1205" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje HET949BSC</t>
         </is>
       </c>
       <c r="E1205" t="n">
@@ -37801,7 +37801,7 @@
       </c>
       <c r="D1206" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG BACKOFENLAMPE,40W, E14</t>
         </is>
       </c>
       <c r="E1206" t="n">
@@ -37863,7 +37863,7 @@
       </c>
       <c r="D1208" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung SD Card PRO Plus (2023) 512GB</t>
         </is>
       </c>
       <c r="E1208" t="n">
@@ -37956,7 +37956,7 @@
       </c>
       <c r="D1211" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko DR 81490</t>
         </is>
       </c>
       <c r="E1211" t="n">
@@ -38049,7 +38049,7 @@
       </c>
       <c r="D1214" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko Aktivkohlenfilter zu CTB6407X/W  9197065088</t>
         </is>
       </c>
       <c r="E1214" t="n">
@@ -38173,7 +38173,7 @@
       </c>
       <c r="D1218" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BIM325GI63DBG Einbau-Mikrowelle mit Grill 25l 900 W</t>
         </is>
       </c>
       <c r="E1218" t="n">
@@ -38235,7 +38235,7 @@
       </c>
       <c r="D1220" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense WF3S8043BW3  Waschmaschine Stand 60cm Frontlader</t>
         </is>
       </c>
       <c r="E1220" t="n">
@@ -38390,7 +38390,7 @@
       </c>
       <c r="D1225" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje ECT641BX Elektrokochfeld 60cm Autark mit Edelstahlrahmen</t>
         </is>
       </c>
       <c r="E1225" t="n">
@@ -38452,7 +38452,7 @@
       </c>
       <c r="D1227" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMI4HTS00E Geschirrspüler Einbau teilintegriert 60cm</t>
         </is>
       </c>
       <c r="E1227" t="n">
@@ -38514,7 +38514,7 @@
       </c>
       <c r="D1229" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate microSDXC 512GB</t>
         </is>
       </c>
       <c r="E1229" t="n">
@@ -38638,7 +38638,7 @@
       </c>
       <c r="D1233" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BBIM12300X Multifunktionsbackrohr mit 8 Kochfunktionen</t>
         </is>
       </c>
       <c r="E1233" t="n">
@@ -38793,7 +38793,7 @@
       </c>
       <c r="D1238" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HVC676451DA Akkustaubsauger 3 in 1 mit All in One Station</t>
         </is>
       </c>
       <c r="E1238" t="n">
@@ -38824,7 +38824,7 @@
       </c>
       <c r="D1239" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 65E8Q</t>
         </is>
       </c>
       <c r="E1239" t="n">
@@ -38979,7 +38979,7 @@
       </c>
       <c r="D1244" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens WG44G2140 iQ500, Waschmaschine, Frontlader, 9 kg, 1400 U/min</t>
         </is>
       </c>
       <c r="E1244" t="n">
@@ -39010,7 +39010,7 @@
       </c>
       <c r="D1245" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens VSP3AAAA Staubsauger mit Beutel,</t>
         </is>
       </c>
       <c r="E1245" t="n">
@@ -39041,7 +39041,7 @@
       </c>
       <c r="D1246" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HI6442BSCE Induktionskochfeld Autark 60cm</t>
         </is>
       </c>
       <c r="E1246" t="n">
@@ -39072,7 +39072,7 @@
       </c>
       <c r="D1247" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch BGC41XSIL Beutelloser Bodenstaubsauger schwarz</t>
         </is>
       </c>
       <c r="E1247" t="n">
@@ -39258,7 +39258,7 @@
       </c>
       <c r="D1253" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S34DG850SU - G85SD Series - OLED-Monitor - Smart - Gaming -</t>
         </is>
       </c>
       <c r="E1253" t="n">
@@ -39785,7 +39785,7 @@
       </c>
       <c r="D1270" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMV6ZCX16E Serie 6, Vollintegrierter Geschirrspüler, 60 cm</t>
         </is>
       </c>
       <c r="E1270" t="n">
@@ -39940,7 +39940,7 @@
       </c>
       <c r="D1275" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung LH85WMBWLGCXEN WM85B, Digitales Flipchart in 85"</t>
         </is>
       </c>
       <c r="E1275" t="n">
@@ -40033,7 +40033,7 @@
       </c>
       <c r="D1278" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje ECS646BCSC Glaskeramik-Kochfeld Autark 60 cm</t>
         </is>
       </c>
       <c r="E1278" t="n">
@@ -40126,7 +40126,7 @@
       </c>
       <c r="D1281" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RF24BB620EB1EF Multi-/French-Door NoFrost</t>
         </is>
       </c>
       <c r="E1281" t="n">
@@ -40188,7 +40188,7 @@
       </c>
       <c r="D1283" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung Odyssey S32DG702EU</t>
         </is>
       </c>
       <c r="E1283" t="n">
@@ -40250,7 +40250,7 @@
       </c>
       <c r="D1285" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje SM703GCB  Kontaktgrill</t>
         </is>
       </c>
       <c r="E1285" t="n">
@@ -40498,7 +40498,7 @@
       </c>
       <c r="D1293" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 65A7Q</t>
         </is>
       </c>
       <c r="E1293" t="n">
@@ -40529,7 +40529,7 @@
       </c>
       <c r="D1294" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S32DG800SU - OLED-Monitor - Smart - Gaming - 80 cm</t>
         </is>
       </c>
       <c r="E1294" t="n">
@@ -40560,7 +40560,7 @@
       </c>
       <c r="D1295" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RF65DG9H0EB1EF 4-Türen French Door mit Family Hub+</t>
         </is>
       </c>
       <c r="E1295" t="n">
@@ -40839,7 +40839,7 @@
       </c>
       <c r="D1304" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 58A6Q</t>
         </is>
       </c>
       <c r="E1304" t="n">
@@ -41025,7 +41025,7 @@
       </c>
       <c r="D1310" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WD90DG5G34BEEG Waschtrockner SLIM 9kg/ 5kg</t>
         </is>
       </c>
       <c r="E1310" t="n">
@@ -41056,7 +41056,7 @@
       </c>
       <c r="D1311" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 55A7Q</t>
         </is>
       </c>
       <c r="E1311" t="n">
@@ -41087,7 +41087,7 @@
       </c>
       <c r="D1312" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate SDXC 256GB</t>
         </is>
       </c>
       <c r="E1312" t="n">
@@ -41242,7 +41242,7 @@
       </c>
       <c r="D1317" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F65KEFEF Side by Side NoFrost 640 Liter</t>
         </is>
       </c>
       <c r="E1317" t="n">
@@ -41304,7 +41304,7 @@
       </c>
       <c r="D1319" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SN43ES22CE  Unterbau-Geschirrspüler</t>
         </is>
       </c>
       <c r="E1319" t="n">
@@ -41459,7 +41459,7 @@
       </c>
       <c r="D1324" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch PKM845F11E Glaskeramik-Kochfeld Autark mit Kochfeldabzug</t>
         </is>
       </c>
       <c r="E1324" t="n">
@@ -41552,7 +41552,7 @@
       </c>
       <c r="D1327" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 40A4S</t>
         </is>
       </c>
       <c r="E1327" t="n">
@@ -41614,7 +41614,7 @@
       </c>
       <c r="D1329" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje H20MOBS4I Stand-Mikrowelle Solo 20l 700W</t>
         </is>
       </c>
       <c r="E1329" t="n">
@@ -41645,7 +41645,7 @@
       </c>
       <c r="D1330" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung USB 3.1 Flash Drive Type-C 512GB</t>
         </is>
       </c>
       <c r="E1330" t="n">
@@ -41707,7 +41707,7 @@
       </c>
       <c r="D1332" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung Sonic the Hedgehog microSDXC 128GB</t>
         </is>
       </c>
       <c r="E1332" t="n">
@@ -41738,7 +41738,7 @@
       </c>
       <c r="D1333" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens TQ903D03 EQ900  Kaffeevollautomat Edelstahl</t>
         </is>
       </c>
       <c r="E1333" t="n">
@@ -41769,7 +41769,7 @@
       </c>
       <c r="D1334" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung SD Card PRO Ultimate 512GB</t>
         </is>
       </c>
       <c r="E1334" t="n">
@@ -41800,7 +41800,7 @@
       </c>
       <c r="D1335" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S32FM700UU</t>
         </is>
       </c>
       <c r="E1335" t="n">
@@ -41862,7 +41862,7 @@
       </c>
       <c r="D1337" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>LG UltraGear 34G600A-B.AEU</t>
         </is>
       </c>
       <c r="E1337" t="n">
@@ -42079,7 +42079,7 @@
       </c>
       <c r="D1344" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RB3B250SAWE Einbau-Kühl-Gefrierkombination</t>
         </is>
       </c>
       <c r="E1344" t="n">
@@ -42141,7 +42141,7 @@
       </c>
       <c r="D1346" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RW3N122GALF Weinkühlschrank</t>
         </is>
       </c>
       <c r="E1346" t="n">
@@ -42234,7 +42234,7 @@
       </c>
       <c r="D1349" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung BAR Plus 256GB</t>
         </is>
       </c>
       <c r="E1349" t="n">
@@ -42265,7 +42265,7 @@
       </c>
       <c r="D1350" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung 43U7020F</t>
         </is>
       </c>
       <c r="E1350" t="n">
@@ -42420,7 +42420,7 @@
       </c>
       <c r="D1355" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate  512GB SD Card  inkl. USB-Kartenleser</t>
         </is>
       </c>
       <c r="E1355" t="n">
@@ -42513,7 +42513,7 @@
       </c>
       <c r="D1358" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung USB Type-C USB 3.2 Gen1 Flash Drive 256 GB</t>
         </is>
       </c>
       <c r="E1358" t="n">
@@ -47876,7 +47876,7 @@
       </c>
       <c r="D1531" t="inlineStr">
         <is>
-          <t>AVM</t>
+          <t>AVM FRITZ!Box 6850 5G</t>
         </is>
       </c>
       <c r="E1531" t="n">
@@ -48155,7 +48155,7 @@
       </c>
       <c r="D1540" t="inlineStr">
         <is>
-          <t>Braun</t>
+          <t>Braun Rasierer Series9 9 9575cc Wet/Dry</t>
         </is>
       </c>
       <c r="E1540" t="n">
@@ -49736,7 +49736,7 @@
       </c>
       <c r="D1591" t="inlineStr">
         <is>
-          <t>Philips</t>
+          <t>Philips HX3603/01 Sonicare for Kids Zahnbürste HX3603/01</t>
         </is>
       </c>
       <c r="E1591" t="n">
@@ -50680,7 +50680,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ProductTitle</t>
+          <t>Product title</t>
         </is>
       </c>
     </row>
@@ -50702,7 +50702,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>Xiaomi Xiaomi Vacuum Cleaner Mi Robot G30 Max Filter Kit EU BHR08C4GL</t>
         </is>
       </c>
     </row>
@@ -50724,7 +50724,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kitchenaid</t>
+          <t>Kitchenaid 5KEK1701EPL Electric Kettle</t>
         </is>
       </c>
     </row>
@@ -50746,7 +50746,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens VZ41AFP Staubsaugerbeutel</t>
         </is>
       </c>
     </row>
@@ -50768,7 +50768,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HEZ431002 Backblech</t>
         </is>
       </c>
     </row>
@@ -50790,7 +50790,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HEZ634000</t>
         </is>
       </c>
     </row>
@@ -50812,7 +50812,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WMZ2381 Verlängerung Wasserzulaufschlauch</t>
         </is>
       </c>
     </row>
@@ -50834,7 +50834,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch TWK4P440 DesignLine</t>
         </is>
       </c>
     </row>
@@ -50856,7 +50856,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje BM201SG3BG  Mikrowelle mit Grill Schwarz</t>
         </is>
       </c>
     </row>
@@ -50878,7 +50878,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI6401BX Kochfeld Induktion 60 cm autark</t>
         </is>
       </c>
     </row>
@@ -50900,7 +50900,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RB49CPW</t>
         </is>
       </c>
     </row>
@@ -50922,7 +50922,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RB49CPW Kühlschrank mit Gefrierfach Stand</t>
         </is>
       </c>
     </row>
@@ -50944,7 +50944,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens LB55565 Lüfterbaustein Silbermetallic</t>
         </is>
       </c>
     </row>
@@ -50966,7 +50966,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WPNF5A84A2TS/AT Waschmaschine Stand 60 cm 8 kg</t>
         </is>
       </c>
     </row>
@@ -50988,7 +50988,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI642E90X Geschirrspüler einbau 60cm teilintegriert</t>
         </is>
       </c>
     </row>
@@ -51010,7 +51010,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW80FG3M05AWEG Waschmaschine 8kg 1400 U/min</t>
         </is>
       </c>
     </row>
@@ -51032,7 +51032,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens LC67BIP50 Wand-Esse Edelstahl 60 cm</t>
         </is>
       </c>
     </row>
@@ -51054,7 +51054,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RL481N4BIE Kühlschrank Stand Inox-Look</t>
         </is>
       </c>
     </row>
@@ -51076,7 +51076,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje JUMP SET AQUA/C  BackofenSet Einbau 60 cm schwarz</t>
         </is>
       </c>
     </row>
@@ -51098,7 +51098,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje NRB620C61X4WFE Kühl-Gefrierkombination Stand</t>
         </is>
       </c>
     </row>
@@ -51120,7 +51120,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WD2PA964ADW/AT Waschtrockner 9 kg Waschen 6 kg Trocknen</t>
         </is>
       </c>
     </row>
@@ -51142,7 +51142,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens EI645CFB6E  Induktions-Kochfeld, 60 cm herdgebunden</t>
         </is>
       </c>
     </row>
@@ -51164,7 +51164,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko HSM46740 Gefriertruhe  451 l</t>
         </is>
       </c>
     </row>
@@ -51186,7 +51186,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch KÜHLSCHRANK INTEG.**** 88X56CM</t>
         </is>
       </c>
     </row>
@@ -51208,7 +51208,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG LAVAMAT L6FBA50490 Waschmaschine Frontlader 9kg</t>
         </is>
       </c>
     </row>
@@ -51230,7 +51230,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FAVORIT FSE73427P</t>
         </is>
       </c>
     </row>
@@ -51252,7 +51252,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SBI4ECS28E Geschirrspüler Einbau teilintegriert 60 cm XXL</t>
         </is>
       </c>
     </row>
@@ -51274,7 +51274,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FSK74747P</t>
         </is>
       </c>
     </row>
@@ -51296,7 +51296,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WASCHVOLLAUTOMAT 9KG 1400UMIN</t>
         </is>
       </c>
     </row>
@@ -51318,7 +51318,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW11DB7B94GEU3 Waschmaschine 11 kg 1400U/Min A-20%</t>
         </is>
       </c>
     </row>
@@ -51340,7 +51340,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WGB244071 Waschmaschine Weiß 9 kg 1400 U/min</t>
         </is>
       </c>
     </row>
@@ -51362,7 +51362,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens HE578BBS3 iQ500, Einbau-Herd, 60 x 60 cm,</t>
         </is>
       </c>
     </row>
@@ -51384,7 +51384,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RQ760N4SASE Side by Side mit Wassertank</t>
         </is>
       </c>
     </row>
@@ -51406,7 +51406,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS68CG852DS9EF Side by Side mit Wassertank NoFrost</t>
         </is>
       </c>
     </row>
@@ -51428,7 +51428,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS80F65KDFEF Side-by-Side  NoFrost 640 Liter</t>
         </is>
       </c>
     </row>
@@ -51450,7 +51450,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung SSD 9100 PRO NVMe 8TB Heatsink</t>
         </is>
       </c>
     </row>
@@ -51472,7 +51472,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG DPGR-AP1 Brat- und Fettpfanne</t>
         </is>
       </c>
     </row>
@@ -51494,7 +51494,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung NK24N1331IS Dunstabzugshaube 60cm Edelstahl</t>
         </is>
       </c>
     </row>
@@ -51516,7 +51516,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WHT6SYB Dekorativ Dunstabzug Kamin 60cm Schwarz</t>
         </is>
       </c>
     </row>
@@ -51538,7 +51538,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens ET601FNP1E Einbau Flächenbündiges Design</t>
         </is>
       </c>
     </row>
@@ -51560,7 +51560,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDIN36432 Geschirrspüler Einbau 60 cm vollintegriert</t>
         </is>
       </c>
     </row>
@@ -51582,7 +51582,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje F49CPW</t>
         </is>
       </c>
     </row>
@@ -51604,7 +51604,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BM3WFT38413W Waschmaschine 1400 U/min 8 kg</t>
         </is>
       </c>
     </row>
@@ -51626,7 +51626,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko B5WFU58416W</t>
         </is>
       </c>
     </row>
@@ -51648,7 +51648,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG L6FBC41480  LAVAMAT Waschmaschinen Frontlader Weiss</t>
         </is>
       </c>
     </row>
@@ -51670,7 +51670,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPV2HKX42E Geschirrspüler Einbau 45 cm vollintegriert</t>
         </is>
       </c>
     </row>
@@ -51692,7 +51692,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HBG578BS3 Backofen Edelstahl Schwarz</t>
         </is>
       </c>
     </row>
@@ -51714,7 +51714,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FSE73407P</t>
         </is>
       </c>
     </row>
@@ -51736,7 +51736,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG FEE7341AZM</t>
         </is>
       </c>
     </row>
@@ -51758,7 +51758,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch KIV86NSE0 Kühl-/Gefrierkombinationen Einbau Weiss</t>
         </is>
       </c>
     </row>
@@ -51780,7 +51780,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMI6ECS12E Teilintegrierter Geschirrspüler, 60 cm, Edelstahl</t>
         </is>
       </c>
     </row>
@@ -51802,7 +51802,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch CBG7341B1 Kompaktbackofen 60x45 EEK: A+</t>
         </is>
       </c>
     </row>
@@ -51824,7 +51824,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch ATMKHERD2 (HEA2130B3 + NKN64RGA2E) Herdset Einbau</t>
         </is>
       </c>
     </row>
@@ -51846,7 +51846,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung QE65S85F 65 Zoll 4K Vision AI TV; OLED TV Schwarz Fernseher</t>
         </is>
       </c>
     </row>
@@ -51868,7 +51868,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS90F64EDFEF Side-by-Side  Premium Black Steel</t>
         </is>
       </c>
     </row>
@@ -51890,7 +51890,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung Sonic the Hedgehog microSDXC 512GB</t>
         </is>
       </c>
     </row>
@@ -51912,7 +51912,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens FF023LMB2 iQ300 Mikrowelle</t>
         </is>
       </c>
     </row>
@@ -51934,7 +51934,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BBIMA13300XS Backofen AirFry 60 cm Schwarz</t>
         </is>
       </c>
     </row>
@@ -51956,7 +51956,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BSA65334ABDG Einbaubackofen schwarz 77 Liter</t>
         </is>
       </c>
     </row>
@@ -51978,7 +51978,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GV663A66  Einbau Geschirrspüler 60cm vollintegriert</t>
         </is>
       </c>
     </row>
@@ -52000,7 +52000,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMS2ITW33E Serie 2 Freistehender Geschirrspüler 60 cm</t>
         </is>
       </c>
     </row>
@@ -52022,7 +52022,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI673B90X Geschirrspüler Einbau 60cm teilintegriert</t>
         </is>
       </c>
     </row>
@@ -52044,7 +52044,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDDN38440XD</t>
         </is>
       </c>
     </row>
@@ -52066,7 +52066,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch GESCHIRRSPÜLER VOLLI.     60CM</t>
         </is>
       </c>
     </row>
@@ -52088,7 +52088,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Electrolux</t>
+          <t>Electrolux LXB3AE82R</t>
         </is>
       </c>
     </row>
@@ -52110,7 +52110,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch KIR21ADD1 Serie 6 Einbau-Kühlschrank ohne Gefrierfach, 88cm</t>
         </is>
       </c>
     </row>
@@ -52132,7 +52132,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje Steel Set 4  BCS6737E06X +  ECD634BCSC</t>
         </is>
       </c>
     </row>
@@ -52154,7 +52154,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens GESCHIRRSPÜLER INTEG.     60CM</t>
         </is>
       </c>
     </row>
@@ -52176,7 +52176,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG LAVAMAT L6FBA51680 Waschmaschine 8 kg 1600 U/min</t>
         </is>
       </c>
     </row>
@@ -52198,7 +52198,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPÜLER TEILINTEGRIERT 60CM</t>
         </is>
       </c>
     </row>
@@ -52220,7 +52220,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SR53HS74KE Geschirrspüler Einbau 45cm teilintegriert</t>
         </is>
       </c>
     </row>
@@ -52242,7 +52242,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WF90F09C4SU3 AI Waschmaschine 9kg 1400 U/min</t>
         </is>
       </c>
     </row>
@@ -52264,7 +52264,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KG39N2XAG Küh-Gefrierkombination  BlackSteel NoFrost</t>
         </is>
       </c>
     </row>
@@ -52286,7 +52286,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KI77SXFE0 iQ500, Einbau-Kühl-Gefrier-Kombination</t>
         </is>
       </c>
     </row>
@@ -52308,7 +52308,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RQ5P605NSVE Multi Door Side-By-Side (4Tür) 591Liter</t>
         </is>
       </c>
     </row>
@@ -52330,7 +52330,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch Bosch Siemens Neff ORIGINAL Lampe  Blau</t>
         </is>
       </c>
     </row>
@@ -52352,7 +52352,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG DUB1611M</t>
         </is>
       </c>
     </row>
@@ -52374,7 +52374,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko CTB 9250 XH Flachschirmhaube Einbau Edelstahl</t>
         </is>
       </c>
     </row>
@@ -52396,7 +52396,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDFN26441W Geschirspüler Stand 6 Programme</t>
         </is>
       </c>
     </row>
@@ -52418,7 +52418,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 55A6Q</t>
         </is>
       </c>
     </row>
@@ -52440,7 +52440,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje NFB612CSXL4  Kühl-Gefrierkombination Stand Nofrost</t>
         </is>
       </c>
     </row>
@@ -52462,7 +52462,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje Jump Induction Set 2 Backofen Set</t>
         </is>
       </c>
     </row>
@@ -52484,7 +52484,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch HBA3140B3 Backofen Schwarz 3D Heißluft</t>
         </is>
       </c>
     </row>
@@ -52506,7 +52506,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense WF5i1245BWR Waschmaschine 12 kg 1400 U/Min.</t>
         </is>
       </c>
     </row>
@@ -52528,7 +52528,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SR43ES25ME Unterbau-Einbau Geschirrspüler 45 cm</t>
         </is>
       </c>
     </row>
@@ -52550,7 +52550,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WAN2820EP Waschmaschine Stand 60 cm weiß</t>
         </is>
       </c>
     </row>
@@ -52572,7 +52572,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG TO64RAF7XB</t>
         </is>
       </c>
     </row>
@@ -52594,7 +52594,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WUU28T48  8kg Frontlader Waschmaschine unterbaufähig</t>
         </is>
       </c>
     </row>
@@ -52616,7 +52616,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko B7T692A3WW  Wärmepumpentrockner 9kg</t>
         </is>
       </c>
     </row>
@@ -52638,7 +52638,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RL5K370GSFC Kühlschrank Stand 372l, Schwarz</t>
         </is>
       </c>
     </row>
@@ -52660,7 +52660,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SN53ES22AE Geschirrspüler Einbau teilintegriert 60 cm</t>
         </is>
       </c>
     </row>
@@ -52682,7 +52682,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens BE732R1B1  iQ700 Einbau-Mikrowelle Schwarz Edelstahl</t>
         </is>
       </c>
     </row>
@@ -52704,7 +52704,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KI42LVFE0 Kühlschrank Einbau 122cm Nische Weiß</t>
         </is>
       </c>
     </row>
@@ -52726,7 +52726,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S27FG810SU - G81SF Series - OLED-Monitor - Gaming - 68.6 cm</t>
         </is>
       </c>
     </row>
@@ -52748,7 +52748,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMI4ECS28E Geschirrspüler Einbau teilintegriert 60 cm</t>
         </is>
       </c>
     </row>
@@ -52770,7 +52770,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Electrolux</t>
+          <t>Electrolux KRB2AE88S</t>
         </is>
       </c>
     </row>
@@ -52792,7 +52792,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDSA250K4SN Einbau Kühl-Gefrierkombination 220 Liter</t>
         </is>
       </c>
     </row>
@@ -52814,7 +52814,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPV2HMX42E Geschirrspüler Einbau vollintegriert 45 cm</t>
         </is>
       </c>
     </row>
@@ -52836,7 +52836,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW90DG5G34AEEG Waschmaschine Slim 9kg ,1400 U/min, 48cm Tief</t>
         </is>
       </c>
     </row>
@@ -52858,7 +52858,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WW1EDG5B25AEEG  Waschmaschine 11 kg 1400 U/min</t>
         </is>
       </c>
     </row>
@@ -52880,7 +52880,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 75E7NQ PRO  75 '' E7N PRO | QLED Smart TV 4K 144 Hz</t>
         </is>
       </c>
     </row>
@@ -52902,7 +52902,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG WASCHMASCHINE TOPL. 6KG  1300U</t>
         </is>
       </c>
     </row>
@@ -52924,7 +52924,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SR65ZX22ME Geschirrspüler Einbau vollintegriert 45cm</t>
         </is>
       </c>
     </row>
@@ -52946,7 +52946,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens EX801KYW1E Einbau Induktion 80cm Edelstahl</t>
         </is>
       </c>
     </row>
@@ -52968,7 +52968,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F64KETEF Side by Side Nofrost  640Liter</t>
         </is>
       </c>
     </row>
@@ -52990,7 +52990,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung COLOR E-PAPER DISPLAY 32ZOLL</t>
         </is>
       </c>
     </row>
@@ -53012,7 +53012,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>LG OLED83C54LA  4K OLED evo Smart TV Fernseher</t>
         </is>
       </c>
     </row>
@@ -53034,7 +53034,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG STAUBBEUTEL F. VAMPYR 5000+</t>
         </is>
       </c>
     </row>
@@ -53056,7 +53056,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje M882528 Filter für WHU</t>
         </is>
       </c>
     </row>
@@ -53078,7 +53078,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje T850DPB Toaster</t>
         </is>
       </c>
     </row>
@@ -53100,7 +53100,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje BHI611ES Lüfterbaustein Montage in Oberschrank</t>
         </is>
       </c>
     </row>
@@ -53122,7 +53122,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje ECT322BCSC/BCSP  Kochfeld 30cm Autark</t>
         </is>
       </c>
     </row>
@@ -53144,7 +53144,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens LU62LFA21 60 cm Weiß   Unterbauhaube</t>
         </is>
       </c>
     </row>
@@ -53166,7 +53166,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GI601FMC Induktionskochfeld 60cm autark</t>
         </is>
       </c>
     </row>
@@ -53188,7 +53188,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje GE5A23WH Stand Herd  50cm</t>
         </is>
       </c>
     </row>
@@ -53210,7 +53210,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch BSS825ALL Unlimited Gen2 Akku-Staubsauger Weiß</t>
         </is>
       </c>
     </row>
@@ -53232,7 +53232,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch PKM675DP1D Kochstelle Glaskeramik 60 cm</t>
         </is>
       </c>
     </row>
@@ -53254,7 +53254,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch MIKROWELLE EINBAU 800W 39X50CM</t>
         </is>
       </c>
     </row>
@@ -53276,7 +53276,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Electrolux</t>
+          <t>Electrolux LUB3AE88S</t>
         </is>
       </c>
     </row>
@@ -53298,7 +53298,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG TSK5O88WDF  Kühlschrank Einbau</t>
         </is>
       </c>
     </row>
@@ -53320,7 +53320,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG TSF5O88WDF</t>
         </is>
       </c>
     </row>
@@ -53342,7 +53342,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens WQ45B2B40  iQ700, Wärmepumpen-Trockner, 9 kg</t>
         </is>
       </c>
     </row>
@@ -53364,7 +53364,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung LS49CG950EUXEN Odyssey Gaming Monitor G95C (49'')</t>
         </is>
       </c>
     </row>
@@ -53386,7 +53386,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung DV90DB7845GEU3  Wärmepumpentrockner 9 kg</t>
         </is>
       </c>
     </row>
@@ -53408,7 +53408,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RF50C530EB1 French Door mit AI NoFrost</t>
         </is>
       </c>
     </row>
@@ -53430,7 +53430,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WRB247C40 Wärmepumpentrockner 9kg</t>
         </is>
       </c>
     </row>
@@ -53452,7 +53452,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F64KDTEF Side by Side NoFrost 640 Liter</t>
         </is>
       </c>
     </row>
@@ -53474,7 +53474,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F64KDFEF Side by Side NoFrost 640 Liter</t>
         </is>
       </c>
     </row>
@@ -53496,7 +53496,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje H23MOBSD1HG Mikrowelle mit Grill,23Liter Schwarz</t>
         </is>
       </c>
     </row>
@@ -53518,7 +53518,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje EC321BCSC Elektrokochfeld 30cm domino</t>
         </is>
       </c>
     </row>
@@ -53540,7 +53540,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDSN26440X Geschirrspüler EInbau teilintegriert 60 cm</t>
         </is>
       </c>
     </row>
@@ -53562,7 +53562,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RK418DPS4WD Kühl-/Gefrierkombination Stand</t>
         </is>
       </c>
     </row>
@@ -53584,7 +53584,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens HB517GBS3 iQ500, Einbau-Backofen, 60 x 60 cm</t>
         </is>
       </c>
     </row>
@@ -53606,7 +53606,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens HE578GBS3 iQ500, Einbau-Herd, 60 x 60 cm,</t>
         </is>
       </c>
     </row>
@@ -53628,7 +53628,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S49DG934SU - G93SD Series - OLED-Monitor - Gaming - gebog</t>
         </is>
       </c>
     </row>
@@ -53650,7 +53650,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG NRN64A06XB</t>
         </is>
       </c>
     </row>
@@ -53672,7 +53672,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HS673A90W Geschirrspüler Stand 60 cm Weiss</t>
         </is>
       </c>
     </row>
@@ -53694,7 +53694,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BSA66334PBDG Einbaubackofen 60cm</t>
         </is>
       </c>
     </row>
@@ -53716,7 +53716,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BI614P8B Einbaubackofen 60cm</t>
         </is>
       </c>
     </row>
@@ -53738,7 +53738,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens KU21RVFE0 Kühlschrank Einbau-Unterbau 82 x 59.8 cm</t>
         </is>
       </c>
     </row>
@@ -53760,7 +53760,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WGG256F7AT Serie 6 Waschmaschine 10 kg, 1600 U/min</t>
         </is>
       </c>
     </row>
@@ -53782,7 +53782,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate microSDXC 256GB</t>
         </is>
       </c>
     </row>
@@ -53804,7 +53804,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje W3NGPI72SBS/AT</t>
         </is>
       </c>
     </row>
@@ -53826,7 +53826,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RI517E41WF Kühlschrank Einbau 178cm Weiss</t>
         </is>
       </c>
     </row>
@@ -53848,7 +53848,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung BRD27713EWW Kühlschrank mit Gefrierfach Festtür 178cm Nische</t>
         </is>
       </c>
     </row>
@@ -53870,7 +53870,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RBI418EE0 Kühlschrank Einbau mit Gefrierfach  178cm Nische</t>
         </is>
       </c>
     </row>
@@ -53892,7 +53892,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje R49CPW Kühlschrank Stand 56cm breit</t>
         </is>
       </c>
     </row>
@@ -53914,7 +53914,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BDSS25N20X Geschirrspüler Einbau 45 cm edeltstahl</t>
         </is>
       </c>
     </row>
@@ -53936,7 +53936,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SPÜLER TEILINTEGRIERT     60CM</t>
         </is>
       </c>
     </row>
@@ -53958,7 +53958,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BFS615S8B  Dampfbackofen Einbau</t>
         </is>
       </c>
     </row>
@@ -53980,7 +53980,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG M3OCD301 Entkalker für Dampfbacköfen 250ml</t>
         </is>
       </c>
     </row>
@@ -54002,7 +54002,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje RBIU609DA1 Unterbau-Einbau Kühlschrank mit Gefrierfach</t>
         </is>
       </c>
     </row>
@@ -54024,7 +54024,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje WPNEI84A1DTS Waschmaschine 8kg 1400 U/min</t>
         </is>
       </c>
     </row>
@@ -54046,7 +54046,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BAS614P8B Einbau Backofen mit Dampffunktion</t>
         </is>
       </c>
     </row>
@@ -54068,7 +54068,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WASCHMASCHINE 1400UPM 7KG 60CM</t>
         </is>
       </c>
     </row>
@@ -54090,7 +54090,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S27D800EAU - S80D Series - LED-Monitor - 68 cm (27")</t>
         </is>
       </c>
     </row>
@@ -54112,7 +54112,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HV693A65UVAD  Geschirrspüler vollintegriert 60 cm</t>
         </is>
       </c>
     </row>
@@ -54134,7 +54134,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WD81TA049BE/EG Waschtrockner 8 kg Waschen 5 kg Trocknen</t>
         </is>
       </c>
     </row>
@@ -54156,7 +54156,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch WAN28094 Waschmaschine 8kg 1400 U/min Weiss</t>
         </is>
       </c>
     </row>
@@ -54178,7 +54178,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch PXX675DC1E Induktionskochfeld Autark 60 cm</t>
         </is>
       </c>
     </row>
@@ -54200,7 +54200,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung DV90F09F4SU3  AI Wärmepumpentrockner 9 kg</t>
         </is>
       </c>
     </row>
@@ -54222,7 +54222,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje B6128B</t>
         </is>
       </c>
     </row>
@@ -54244,7 +54244,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje HET949BSC</t>
         </is>
       </c>
     </row>
@@ -54266,7 +54266,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>AEG</t>
+          <t>AEG BACKOFENLAMPE,40W, E14</t>
         </is>
       </c>
     </row>
@@ -54288,7 +54288,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung SD Card PRO Plus (2023) 512GB</t>
         </is>
       </c>
     </row>
@@ -54310,7 +54310,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko DR 81490</t>
         </is>
       </c>
     </row>
@@ -54332,7 +54332,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko Aktivkohlenfilter zu CTB6407X/W  9197065088</t>
         </is>
       </c>
     </row>
@@ -54354,7 +54354,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense BIM325GI63DBG Einbau-Mikrowelle mit Grill 25l 900 W</t>
         </is>
       </c>
     </row>
@@ -54376,7 +54376,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense WF3S8043BW3  Waschmaschine Stand 60cm Frontlader</t>
         </is>
       </c>
     </row>
@@ -54398,7 +54398,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje ECT641BX Elektrokochfeld 60cm Autark mit Edelstahlrahmen</t>
         </is>
       </c>
     </row>
@@ -54420,7 +54420,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMI4HTS00E Geschirrspüler Einbau teilintegriert 60cm</t>
         </is>
       </c>
     </row>
@@ -54442,7 +54442,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate microSDXC 512GB</t>
         </is>
       </c>
     </row>
@@ -54464,7 +54464,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Beko</t>
+          <t>Beko BBIM12300X Multifunktionsbackrohr mit 8 Kochfunktionen</t>
         </is>
       </c>
     </row>
@@ -54486,7 +54486,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HVC676451DA Akkustaubsauger 3 in 1 mit All in One Station</t>
         </is>
       </c>
     </row>
@@ -54508,7 +54508,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 65E8Q</t>
         </is>
       </c>
     </row>
@@ -54530,7 +54530,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens WG44G2140 iQ500, Waschmaschine, Frontlader, 9 kg, 1400 U/min</t>
         </is>
       </c>
     </row>
@@ -54552,7 +54552,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens VSP3AAAA Staubsauger mit Beutel,</t>
         </is>
       </c>
     </row>
@@ -54574,7 +54574,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense HI6442BSCE Induktionskochfeld Autark 60cm</t>
         </is>
       </c>
     </row>
@@ -54596,7 +54596,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch BGC41XSIL Beutelloser Bodenstaubsauger schwarz</t>
         </is>
       </c>
     </row>
@@ -54618,7 +54618,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S34DG850SU - G85SD Series - OLED-Monitor - Smart - Gaming -</t>
         </is>
       </c>
     </row>
@@ -54640,7 +54640,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch SMV6ZCX16E Serie 6, Vollintegrierter Geschirrspüler, 60 cm</t>
         </is>
       </c>
     </row>
@@ -54662,7 +54662,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung LH85WMBWLGCXEN WM85B, Digitales Flipchart in 85"</t>
         </is>
       </c>
     </row>
@@ -54684,7 +54684,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje ECS646BCSC Glaskeramik-Kochfeld Autark 60 cm</t>
         </is>
       </c>
     </row>
@@ -54706,7 +54706,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RF24BB620EB1EF Multi-/French-Door NoFrost</t>
         </is>
       </c>
     </row>
@@ -54728,7 +54728,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung Odyssey S32DG702EU</t>
         </is>
       </c>
     </row>
@@ -54750,7 +54750,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje SM703GCB  Kontaktgrill</t>
         </is>
       </c>
     </row>
@@ -54772,7 +54772,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 65A7Q</t>
         </is>
       </c>
     </row>
@@ -54794,7 +54794,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S32DG800SU - OLED-Monitor - Smart - Gaming - 80 cm</t>
         </is>
       </c>
     </row>
@@ -54816,7 +54816,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RF65DG9H0EB1EF 4-Türen French Door mit Family Hub+</t>
         </is>
       </c>
     </row>
@@ -54838,7 +54838,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 58A6Q</t>
         </is>
       </c>
     </row>
@@ -54860,7 +54860,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung WD90DG5G34BEEG Waschtrockner SLIM 9kg/ 5kg</t>
         </is>
       </c>
     </row>
@@ -54882,7 +54882,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 55A7Q</t>
         </is>
       </c>
     </row>
@@ -54904,7 +54904,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate SDXC 256GB</t>
         </is>
       </c>
     </row>
@@ -54926,7 +54926,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung RS70F65KEFEF Side by Side NoFrost 640 Liter</t>
         </is>
       </c>
     </row>
@@ -54948,7 +54948,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens SN43ES22CE  Unterbau-Geschirrspüler</t>
         </is>
       </c>
     </row>
@@ -54970,7 +54970,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Bosch PKM845F11E Glaskeramik-Kochfeld Autark mit Kochfeldabzug</t>
         </is>
       </c>
     </row>
@@ -54992,7 +54992,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense 40A4S</t>
         </is>
       </c>
     </row>
@@ -55014,7 +55014,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Gorenje</t>
+          <t>Gorenje H20MOBS4I Stand-Mikrowelle Solo 20l 700W</t>
         </is>
       </c>
     </row>
@@ -55036,7 +55036,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung USB 3.1 Flash Drive Type-C 512GB</t>
         </is>
       </c>
     </row>
@@ -55058,7 +55058,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung Sonic the Hedgehog microSDXC 128GB</t>
         </is>
       </c>
     </row>
@@ -55080,7 +55080,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Siemens TQ903D03 EQ900  Kaffeevollautomat Edelstahl</t>
         </is>
       </c>
     </row>
@@ -55102,7 +55102,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung SD Card PRO Ultimate 512GB</t>
         </is>
       </c>
     </row>
@@ -55124,7 +55124,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung S32FM700UU</t>
         </is>
       </c>
     </row>
@@ -55146,7 +55146,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>LG UltraGear 34G600A-B.AEU</t>
         </is>
       </c>
     </row>
@@ -55168,7 +55168,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RB3B250SAWE Einbau-Kühl-Gefrierkombination</t>
         </is>
       </c>
     </row>
@@ -55190,7 +55190,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Hisense</t>
+          <t>Hisense RW3N122GALF Weinkühlschrank</t>
         </is>
       </c>
     </row>
@@ -55212,7 +55212,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung BAR Plus 256GB</t>
         </is>
       </c>
     </row>
@@ -55234,7 +55234,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung 43U7020F</t>
         </is>
       </c>
     </row>
@@ -55256,7 +55256,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung PRO Ultimate  512GB SD Card  inkl. USB-Kartenleser</t>
         </is>
       </c>
     </row>
@@ -55278,7 +55278,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Samsung USB Type-C USB 3.2 Gen1 Flash Drive 256 GB</t>
         </is>
       </c>
     </row>
@@ -55300,7 +55300,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>AVM</t>
+          <t>AVM FRITZ!Box 6850 5G</t>
         </is>
       </c>
     </row>
@@ -55322,7 +55322,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Braun</t>
+          <t>Braun Rasierer Series9 9 9575cc Wet/Dry</t>
         </is>
       </c>
     </row>
@@ -55344,7 +55344,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Philips</t>
+          <t>Philips HX3603/01 Sonicare for Kids Zahnbürste HX3603/01</t>
         </is>
       </c>
     </row>

</xml_diff>